<commit_message>
add 12B data to figures 1, 2, and 4; checkpoint integration rewrite
- Fix fig1 bug: behavioral data and loop range now match 5-model MODELS list
- Add 12B behavioral scores derived from perplexity ratios to fig1
- Correct 12B total layers from 40 to 36 in fig1
- Add 12B perplexity data (screen_reader, alt_text, skip_link) to CSV and fig2
- Deprecate generate-figures.py in favor of individual fig scripts
- Include paper section restructuring, extended notebooks, and build updates

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/accessibility-knowledge-emergence/results/analysis/AttentionBindingPythiaModels-ClaudeInExcel.xlsx
+++ b/accessibility-knowledge-emergence/results/analysis/AttentionBindingPythiaModels-ClaudeInExcel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/trishasalas/Repos/Research/how-models-think/accessibility-knowledge-emergence/results/analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10FCDC74-43D0-E549-B254-7ABE56F5CBA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F22CFAE-9D4B-494D-A79A-71BC3266D1DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17180" xr2:uid="{81DF49B0-1BA3-D947-B774-10FF709E1CBE}"/>
+    <workbookView xWindow="38400" yWindow="600" windowWidth="38400" windowHeight="21000" activeTab="7" xr2:uid="{81DF49B0-1BA3-D947-B774-10FF709E1CBE}"/>
   </bookViews>
   <sheets>
     <sheet name="Claude Log" sheetId="12" r:id="rId1"/>

</xml_diff>